<commit_message>
fix: excel fayllaridagi barcha cell note (izohlar) to'liq olib tashlandi, faqat sonlar va formulalar qoldirildi
</commit_message>
<xml_diff>
--- a/DAVOMAT.xlsx
+++ b/DAVOMAT.xlsx
@@ -15,179 +15,6 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Author</author>
-  </authors>
-  <commentList>
-    <comment ref="E4" authorId="0">
-      <text>
-        <r>
-          <t>Inspektor: Rejalashtirilgan ochiq dars</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M4" authorId="0">
-      <text>
-        <r>
-          <t>Inspektor: API verification check</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Y4" authorId="0">
-      <text>
-        <r>
-          <t>Inspektor: Sinov davomati</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Z4" authorId="0">
-      <text>
-        <r>
-          <t>Inspektor: 2-para davomati</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M5" authorId="0">
-      <text>
-        <r>
-          <t>Inspektor Aliyev: 1 talaba betob</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M7" authorId="0">
-      <text>
-        <r>
-          <t>Inspektor Aliyev: A'lo davomat</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M8" authorId="0">
-      <text>
-        <r>
-          <t>Inspektor Aliyev: Barcha talabalar joyida</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N9" authorId="0">
-      <text>
-        <r>
-          <t>Nazoratchi Karimova: 2 talaba sababli</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N11" authorId="0">
-      <text>
-        <r>
-          <t>Nazoratchi Karimova: Kompyuter sinfida amaliy dars</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Author</author>
-  </authors>
-  <commentList>
-    <comment ref="F4" authorId="0">
-      <text>
-        <r>
-          <t>Uslubchi: efgasfgar</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Q4" authorId="0">
-      <text>
-        <r>
-          <t>Inspektor: A'lo qatnashish</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AA6" authorId="0">
-      <text>
-        <r>
-          <t>Uslubchi (Filologiya): malaka oshirshda</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Author</author>
-  </authors>
-  <commentList>
-    <comment ref="G4" authorId="0">
-      <text>
-        <r>
-          <t>Uslubchi: sdgasdfAGFG</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N4" authorId="0">
-      <text>
-        <r>
-          <t>Nazoratchi Karimova: 2 talaba uzrli</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G7" authorId="0">
-      <text>
-        <r>
-          <t>Uslubchi: sdgasdfAGFGAFGA</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G13" authorId="0">
-      <text>
-        <r>
-          <t>Uslubchi: sdgasdfAGFGAFGA</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G32" authorId="0">
-      <text>
-        <r>
-          <t>Uslubchi: sdgasdfAGFGAFGA</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Author</author>
-  </authors>
-  <commentList>
-    <comment ref="N6" authorId="0">
-      <text>
-        <r>
-          <t>Nazoratchi Karimova: Laboratoriya mashg'uloti</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M9" authorId="0">
-      <text>
-        <r>
-          <t>Inspektor Aliyev: 1 talaba kechikib keldi</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="275">
   <si>
@@ -949,7 +776,7 @@
     <t>URGANCH DAVLAT PEDAGOGIKA INSTITUTI (UrDPI) - UMUMIY DAVOMAT MONITORINGI</t>
   </si>
   <si>
-    <t>Oxirgi yangilanish: 19/10/2026, 14:54:12 | Barcha 5 ta fakultet bo'yicha integratsiyalangan hisobot</t>
+    <t>Oxirgi yangilanish: 19/10/2026, 15:13:23 | Barcha 5 ta fakultet bo'yicha integratsiyalangan hisobot</t>
   </si>
   <si>
     <t>№</t>
@@ -2925,7 +2752,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -5552,7 +5378,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -7300,7 +7125,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -10362,7 +10186,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Auditoriya va Tekshiruvchi maydonlarini soddalashtirish, Telegram bot va auditorlar tizimini yangilash
</commit_message>
<xml_diff>
--- a/DAVOMAT.xlsx
+++ b/DAVOMAT.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="276">
   <si>
     <t>ANIQ FANLAR OLIY MAKTABI - KUNDUZGI YO'NALISHLAR DAVOMAT JADVALI</t>
   </si>
@@ -776,7 +776,7 @@
     <t>URGANCH DAVLAT PEDAGOGIKA INSTITUTI (UrDPI) - UMUMIY DAVOMAT MONITORINGI</t>
   </si>
   <si>
-    <t>Oxirgi yangilanish: 19/10/2026, 15:13:23 | Barcha 5 ta fakultet bo'yicha integratsiyalangan hisobot</t>
+    <t>Oxirgi yangilanish: 21/10/2026, 10:28:10 | Barcha 5 ta fakultet bo'yicha integratsiyalangan hisobot</t>
   </si>
   <si>
     <t>№</t>
@@ -803,22 +803,25 @@
     <t>Holat</t>
   </si>
   <si>
-    <t>97.0%</t>
-  </si>
-  <si>
-    <t>94.2%</t>
+    <t>94.7%</t>
+  </si>
+  <si>
+    <t>95.2%</t>
   </si>
   <si>
     <t>A'lo</t>
   </si>
   <si>
-    <t>96.2%</t>
-  </si>
-  <si>
-    <t>98.7%</t>
-  </si>
-  <si>
-    <t>97.1%</t>
+    <t>88.5%</t>
+  </si>
+  <si>
+    <t>97.9%</t>
+  </si>
+  <si>
+    <t>Yaxshi</t>
+  </si>
+  <si>
+    <t>113.0%</t>
   </si>
   <si>
     <t>97.6%</t>
@@ -830,7 +833,7 @@
     <t>Kutilmoqda</t>
   </si>
   <si>
-    <t>100.0%</t>
+    <t>110.9%</t>
   </si>
   <si>
     <t>98.8%</t>
@@ -839,7 +842,7 @@
     <t>INSTITUT BO'YICHA JAMI</t>
   </si>
   <si>
-    <t>97.4%</t>
+    <t>97.5%</t>
   </si>
   <si>
     <t>Barqaror</t>
@@ -852,7 +855,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -904,6 +907,10 @@
       <color rgb="FF16A34A"/>
     </font>
     <font>
+      <b/>
+      <color rgb="FF2563EB"/>
+    </font>
+    <font>
       <i/>
       <color rgb="FF94A3B8"/>
     </font>
@@ -946,7 +953,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -989,13 +996,16 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1499,18 +1509,21 @@
         <v>24</v>
       </c>
       <c r="H4" s="6">
-        <f t="shared" ref="H4:H34" si="2">IFERROR(AVERAGE(E4:G4)/D4,"")</f>
+        <f t="shared" ref="H4:H34" si="0">IFERROR(AVERAGE(E4:G4)/D4,"")</f>
         <v>0.96</v>
       </c>
       <c r="L4" s="6">
-        <f t="shared" ref="L4:L35" si="0">IFERROR(AVERAGE(I4:K4)/D4,"")</f>
+        <f t="shared" ref="L4:L35" si="1">IFERROR(AVERAGE(I4:K4)/D4,"")</f>
       </c>
       <c r="M4" s="5">
         <v>24</v>
       </c>
+      <c r="N4" s="5">
+        <v>25</v>
+      </c>
       <c r="P4" s="6">
-        <f t="shared" ref="P4:P34" si="5">IFERROR(AVERAGE(M4:O4)/D4,"")</f>
-        <v>0.96</v>
+        <f t="shared" ref="P4:P34" si="2">IFERROR(AVERAGE(M4:O4)/D4,"")</f>
+        <v>0.98</v>
       </c>
       <c r="R4" s="5">
         <v>24</v>
@@ -1523,7 +1536,7 @@
         <v>0.9</v>
       </c>
       <c r="X4" s="6">
-        <f t="shared" ref="X4:X35" si="1">IFERROR(AVERAGE(U4:W4)/D4,"")</f>
+        <f t="shared" ref="X4:X35" si="4">IFERROR(AVERAGE(U4:W4)/D4,"")</f>
       </c>
       <c r="Y4" s="5">
         <v>24</v>
@@ -1532,12 +1545,12 @@
         <v>24</v>
       </c>
       <c r="AB4" s="6">
-        <f t="shared" ref="AB4:AB34" si="4">IFERROR(AVERAGE(Y4:AA4)/D4,"")</f>
+        <f t="shared" ref="AB4:AB34" si="5">IFERROR(AVERAGE(Y4:AA4)/D4,"")</f>
         <v>0.96</v>
       </c>
       <c r="AC4" s="6">
         <f t="shared" ref="AC4:AC34" si="6">IFERROR(AVERAGE(H4,L4,P4,T4,X4,AB4),"")</f>
-        <v>0.945</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.25">
@@ -1554,10 +1567,10 @@
         <v>22</v>
       </c>
       <c r="H5" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L5" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="M5" s="5">
         <v>21</v>
@@ -1570,10 +1583,10 @@
         <f t="shared" si="3"/>
       </c>
       <c r="X5" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB5" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC5" s="6">
         <f>IFERROR(AVERAGE(H5,L5,P5,T5,X5,AB5),"")</f>
@@ -1601,20 +1614,20 @@
         <v>1</v>
       </c>
       <c r="L6" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="O6" s="5"/>
       <c r="P6" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T6" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X6" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB6" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC6" s="6">
         <f>IFERROR(AVERAGE(H6,L6,P6,T6,X6,AB6),"")</f>
@@ -1635,12 +1648,15 @@
         <v>26</v>
       </c>
       <c r="H7" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L7" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="M7" s="5">
+        <v>26</v>
+      </c>
+      <c r="N7" s="5">
         <v>26</v>
       </c>
       <c r="P7" s="6">
@@ -1651,10 +1667,10 @@
         <f t="shared" si="3"/>
       </c>
       <c r="X7" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB7" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC7" s="6">
         <f>IFERROR(AVERAGE(H7,L7,P7,T7,X7,AB7),"")</f>
@@ -1675,10 +1691,10 @@
         <v>28</v>
       </c>
       <c r="H8" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L8" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="M8" s="5">
         <v>24</v>
@@ -1691,10 +1707,10 @@
         <f t="shared" si="3"/>
       </c>
       <c r="X8" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB8" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC8" s="6">
         <f>IFERROR(AVERAGE(H8,L8,P8,T8,X8,AB8),"")</f>
@@ -1715,10 +1731,10 @@
         <v>26</v>
       </c>
       <c r="H9" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L9" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="N9" s="5">
         <v>24</v>
@@ -1731,10 +1747,10 @@
         <f t="shared" si="3"/>
       </c>
       <c r="X9" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB9" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC9" s="6">
         <f>IFERROR(AVERAGE(H9,L9,P9,T9,X9,AB9),"")</f>
@@ -1755,22 +1771,22 @@
         <v>25</v>
       </c>
       <c r="H10" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L10" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P10" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T10" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X10" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB10" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC10" s="6">
         <f t="shared" si="6"/>
@@ -1790,10 +1806,10 @@
         <v>22</v>
       </c>
       <c r="H11" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L11" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="N11" s="5">
         <v>22</v>
@@ -1806,10 +1822,10 @@
         <f t="shared" si="3"/>
       </c>
       <c r="X11" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB11" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC11" s="6">
         <f>IFERROR(AVERAGE(H11,L11,P11,T11,X11,AB11),"")</f>
@@ -1830,22 +1846,22 @@
         <v>22</v>
       </c>
       <c r="H12" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L12" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P12" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T12" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X12" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB12" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC12" s="6">
         <f t="shared" si="6"/>
@@ -1865,10 +1881,10 @@
         <v>19</v>
       </c>
       <c r="H13" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L13" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="M13" s="5"/>
       <c r="O13" s="5">
@@ -1882,10 +1898,10 @@
         <f t="shared" si="3"/>
       </c>
       <c r="X13" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB13" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC13" s="6">
         <f>IFERROR(AVERAGE(H13,L13,P13,T13,X13,AB13),"")</f>
@@ -1906,23 +1922,23 @@
         <v>19</v>
       </c>
       <c r="H14" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L14" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="M14" s="5"/>
       <c r="P14" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T14" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X14" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB14" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC14" s="6">
         <f t="shared" si="6"/>
@@ -1942,10 +1958,10 @@
         <v>26</v>
       </c>
       <c r="H15" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L15" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="O15" s="5">
         <v>23</v>
@@ -1958,10 +1974,10 @@
         <f t="shared" si="3"/>
       </c>
       <c r="X15" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB15" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC15" s="6">
         <f>IFERROR(AVERAGE(H15,L15,P15,T15,X15,AB15),"")</f>
@@ -1982,25 +1998,30 @@
         <v>26</v>
       </c>
       <c r="H16" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L16" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
+      </c>
+      <c r="N16" s="5">
+        <v>26</v>
       </c>
       <c r="P16" s="6">
-        <f t="shared" si="5"/>
+        <f>IFERROR(AVERAGE(M16:O16)/D16,"")</f>
+        <v>1</v>
       </c>
       <c r="T16" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X16" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB16" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC16" s="6">
-        <f t="shared" si="6"/>
+        <f>IFERROR(AVERAGE(H16,L16,P16,T16,X16,AB16),"")</f>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:29" x14ac:dyDescent="0.25">
@@ -2017,22 +2038,22 @@
         <v>13</v>
       </c>
       <c r="H17" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L17" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P17" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T17" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X17" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB17" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC17" s="6">
         <f t="shared" si="6"/>
@@ -2052,23 +2073,23 @@
         <v>21</v>
       </c>
       <c r="H18" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L18" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="O18" s="5"/>
       <c r="P18" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T18" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X18" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB18" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC18" s="6">
         <f t="shared" si="6"/>
@@ -2088,22 +2109,22 @@
         <v>23</v>
       </c>
       <c r="H19" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L19" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P19" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T19" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X19" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB19" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC19" s="6">
         <f t="shared" si="6"/>
@@ -2123,22 +2144,22 @@
         <v>22</v>
       </c>
       <c r="H20" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L20" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P20" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T20" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X20" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB20" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC20" s="6">
         <f t="shared" si="6"/>
@@ -2158,23 +2179,23 @@
         <v>27</v>
       </c>
       <c r="H21" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L21" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="N21" s="5"/>
       <c r="P21" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T21" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X21" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB21" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC21" s="6">
         <f t="shared" si="6"/>
@@ -2194,22 +2215,22 @@
         <v>27</v>
       </c>
       <c r="H22" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L22" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P22" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T22" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X22" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB22" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC22" s="6">
         <f t="shared" si="6"/>
@@ -2229,25 +2250,30 @@
         <v>21</v>
       </c>
       <c r="H23" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
+      </c>
+      <c r="I23" s="5">
+        <v>21</v>
       </c>
       <c r="L23" s="6">
-        <f t="shared" si="0"/>
+        <f>IFERROR(AVERAGE(I23:K23)/D23,"")</f>
+        <v>1</v>
       </c>
       <c r="P23" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T23" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X23" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB23" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC23" s="6">
-        <f t="shared" si="6"/>
+        <f>IFERROR(AVERAGE(H23,L23,P23,T23,X23,AB23),"")</f>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:29" x14ac:dyDescent="0.25">
@@ -2264,25 +2290,30 @@
         <v>21</v>
       </c>
       <c r="H24" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L24" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
+      </c>
+      <c r="N24" s="5">
+        <v>20</v>
       </c>
       <c r="P24" s="6">
-        <f t="shared" si="5"/>
+        <f>IFERROR(AVERAGE(M24:O24)/D24,"")</f>
+        <v>0.9524</v>
       </c>
       <c r="T24" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X24" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB24" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC24" s="6">
-        <f t="shared" si="6"/>
+        <f>IFERROR(AVERAGE(H24,L24,P24,T24,X24,AB24),"")</f>
+        <v>0.9524</v>
       </c>
     </row>
     <row r="25" spans="1:29" x14ac:dyDescent="0.25">
@@ -2299,22 +2330,22 @@
         <v>11</v>
       </c>
       <c r="H25" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L25" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P25" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T25" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X25" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB25" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC25" s="6">
         <f t="shared" si="6"/>
@@ -2334,10 +2365,10 @@
         <v>21</v>
       </c>
       <c r="H26" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L26" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="N26" s="5"/>
       <c r="O26" s="5">
@@ -2351,10 +2382,10 @@
         <f t="shared" si="3"/>
       </c>
       <c r="X26" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB26" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC26" s="6">
         <f>IFERROR(AVERAGE(H26,L26,P26,T26,X26,AB26),"")</f>
@@ -2375,22 +2406,22 @@
         <v>21</v>
       </c>
       <c r="H27" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L27" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P27" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T27" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X27" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB27" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC27" s="6">
         <f t="shared" si="6"/>
@@ -2410,23 +2441,23 @@
         <v>22</v>
       </c>
       <c r="H28" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L28" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="O28" s="5"/>
       <c r="P28" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T28" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X28" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB28" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC28" s="6">
         <f t="shared" si="6"/>
@@ -2446,22 +2477,22 @@
         <v>28</v>
       </c>
       <c r="H29" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L29" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P29" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T29" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X29" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB29" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC29" s="6">
         <f t="shared" si="6"/>
@@ -2481,22 +2512,22 @@
         <v>22</v>
       </c>
       <c r="H30" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L30" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P30" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T30" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X30" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB30" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC30" s="6">
         <f t="shared" si="6"/>
@@ -2516,22 +2547,22 @@
         <v>24</v>
       </c>
       <c r="H31" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L31" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P31" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T31" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X31" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB31" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC31" s="6">
         <f t="shared" si="6"/>
@@ -2551,22 +2582,22 @@
         <v>24</v>
       </c>
       <c r="H32" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L32" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P32" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T32" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X32" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB32" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC32" s="6">
         <f t="shared" si="6"/>
@@ -2586,22 +2617,22 @@
         <v>27</v>
       </c>
       <c r="H33" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L33" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P33" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T33" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X33" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB33" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC33" s="6">
         <f t="shared" si="6"/>
@@ -2621,22 +2652,22 @@
         <v>27</v>
       </c>
       <c r="H34" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L34" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P34" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T34" s="6">
         <f t="shared" si="3"/>
       </c>
       <c r="X34" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB34" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC34" s="6">
         <f t="shared" si="6"/>
@@ -2667,6 +2698,7 @@
       </c>
       <c r="I35">
         <f>SUM(I4:I34)</f>
+        <v>21</v>
       </c>
       <c r="J35">
         <f>SUM(J4:J34)</f>
@@ -2675,7 +2707,8 @@
         <f>SUM(K4:K34)</f>
       </c>
       <c r="L35" s="6">
-        <f t="shared" si="0"/>
+        <f>IFERROR(AVERAGE(I35:K35)/D35,"")</f>
+        <v>0.0302</v>
       </c>
       <c r="M35">
         <f>SUM(M4:M34)</f>
@@ -2683,7 +2716,7 @@
       </c>
       <c r="N35">
         <f>SUM(N4:N34)</f>
-        <v>46</v>
+        <v>143</v>
       </c>
       <c r="O35">
         <f>SUM(O4:O34)</f>
@@ -2691,7 +2724,7 @@
       </c>
       <c r="P35" s="6">
         <f>IFERROR(AVERAGE(M35:O35)/D35,"")</f>
-        <v>0.0963</v>
+        <v>0.1427</v>
       </c>
       <c r="Q35">
         <f>SUM(Q4:Q34)</f>
@@ -2718,7 +2751,7 @@
         <f>SUM(W4:W34)</f>
       </c>
       <c r="X35" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="Y35">
         <f>SUM(Y4:Y34)</f>
@@ -2737,7 +2770,7 @@
       </c>
       <c r="AC35" s="6">
         <f>IFERROR(AVERAGE(H35,L35,P35,T35,X35,AB35),"")</f>
-        <v>0.0508</v>
+        <v>0.056</v>
       </c>
     </row>
   </sheetData>
@@ -2913,16 +2946,20 @@
         <v>25</v>
       </c>
       <c r="H4" s="6">
-        <f t="shared" ref="H4:H29" si="4">IFERROR(AVERAGE(E4:G4)/D4,"")</f>
+        <f t="shared" ref="H4:H29" si="3">IFERROR(AVERAGE(E4:G4)/D4,"")</f>
         <v>0.9615</v>
       </c>
       <c r="L4" s="6">
         <f t="shared" ref="L4:L30" si="0">IFERROR(AVERAGE(I4:K4)/D4,"")</f>
       </c>
       <c r="M4" s="5"/>
+      <c r="N4" s="5">
+        <v>23</v>
+      </c>
       <c r="O4" s="5"/>
       <c r="P4" s="6">
-        <f t="shared" ref="P4:P35" si="1">IFERROR(AVERAGE(M4:O4)/D4,"")</f>
+        <f t="shared" ref="P4:P30" si="4">IFERROR(AVERAGE(M4:O4)/D4,"")</f>
+        <v>0.8846</v>
       </c>
       <c r="Q4" s="5">
         <v>25</v>
@@ -2932,14 +2969,14 @@
         <v>0.9615</v>
       </c>
       <c r="X4" s="6">
-        <f t="shared" ref="X4:X35" si="2">IFERROR(AVERAGE(U4:W4)/D4,"")</f>
+        <f t="shared" ref="X4:X35" si="1">IFERROR(AVERAGE(U4:W4)/D4,"")</f>
       </c>
       <c r="AB4" s="6">
-        <f t="shared" ref="AB4:AB35" si="3">IFERROR(AVERAGE(Y4:AA4)/D4,"")</f>
+        <f t="shared" ref="AB4:AB35" si="2">IFERROR(AVERAGE(Y4:AA4)/D4,"")</f>
       </c>
       <c r="AC4" s="6">
         <f t="shared" ref="AC4:AC35" si="6">IFERROR(AVERAGE(H4,L4,P4,T4,X4,AB4),"")</f>
-        <v>0.9615</v>
+        <v>0.9359</v>
       </c>
     </row>
     <row r="5" spans="2:29" x14ac:dyDescent="0.25">
@@ -2953,7 +2990,7 @@
         <v>18</v>
       </c>
       <c r="H5" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L5" s="6">
         <f t="shared" si="0"/>
@@ -2961,16 +2998,16 @@
       <c r="M5" s="5"/>
       <c r="O5" s="5"/>
       <c r="P5" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T5" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X5" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB5" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC5" s="6">
         <f t="shared" si="6"/>
@@ -2987,7 +3024,7 @@
         <v>31</v>
       </c>
       <c r="H6" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L6" s="6">
         <f t="shared" si="0"/>
@@ -2995,13 +3032,13 @@
       <c r="M6" s="5"/>
       <c r="O6" s="5"/>
       <c r="P6" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T6" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X6" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AA6" s="5">
         <v>31</v>
@@ -3026,7 +3063,7 @@
         <v>27</v>
       </c>
       <c r="H7" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L7" s="6">
         <f t="shared" si="0"/>
@@ -3034,16 +3071,16 @@
       <c r="M7" s="5"/>
       <c r="O7" s="5"/>
       <c r="P7" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T7" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X7" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB7" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC7" s="6">
         <f t="shared" si="6"/>
@@ -3060,7 +3097,7 @@
         <v>24</v>
       </c>
       <c r="H8" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L8" s="6">
         <f t="shared" si="0"/>
@@ -3068,16 +3105,16 @@
       <c r="M8" s="5"/>
       <c r="O8" s="5"/>
       <c r="P8" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T8" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X8" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB8" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC8" s="6">
         <f t="shared" si="6"/>
@@ -3094,7 +3131,7 @@
         <v>18</v>
       </c>
       <c r="H9" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L9" s="6">
         <f t="shared" si="0"/>
@@ -3102,13 +3139,13 @@
       <c r="M9" s="5"/>
       <c r="O9" s="5"/>
       <c r="P9" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T9" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X9" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AA9" s="5">
         <v>18</v>
@@ -3133,7 +3170,7 @@
         <v>16</v>
       </c>
       <c r="H10" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L10" s="6">
         <f t="shared" si="0"/>
@@ -3141,16 +3178,16 @@
       <c r="M10" s="5"/>
       <c r="O10" s="5"/>
       <c r="P10" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T10" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X10" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB10" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC10" s="6">
         <f t="shared" si="6"/>
@@ -3167,7 +3204,7 @@
         <v>15</v>
       </c>
       <c r="H11" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L11" s="6">
         <f t="shared" si="0"/>
@@ -3175,16 +3212,16 @@
       <c r="M11" s="5"/>
       <c r="O11" s="5"/>
       <c r="P11" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T11" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X11" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB11" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC11" s="6">
         <f t="shared" si="6"/>
@@ -3201,7 +3238,7 @@
         <v>12</v>
       </c>
       <c r="H12" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L12" s="6">
         <f t="shared" si="0"/>
@@ -3209,16 +3246,16 @@
       <c r="M12" s="5"/>
       <c r="O12" s="5"/>
       <c r="P12" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T12" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X12" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB12" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC12" s="6">
         <f t="shared" si="6"/>
@@ -3235,7 +3272,7 @@
         <v>14</v>
       </c>
       <c r="H13" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L13" s="6">
         <f t="shared" si="0"/>
@@ -3243,16 +3280,16 @@
       <c r="M13" s="5"/>
       <c r="O13" s="5"/>
       <c r="P13" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T13" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X13" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB13" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC13" s="6">
         <f t="shared" si="6"/>
@@ -3269,7 +3306,7 @@
         <v>17</v>
       </c>
       <c r="H14" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L14" s="6">
         <f t="shared" si="0"/>
@@ -3277,16 +3314,16 @@
       <c r="M14" s="5"/>
       <c r="O14" s="5"/>
       <c r="P14" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T14" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X14" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB14" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC14" s="6">
         <f t="shared" si="6"/>
@@ -3303,7 +3340,7 @@
         <v>15</v>
       </c>
       <c r="H15" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L15" s="6">
         <f t="shared" si="0"/>
@@ -3311,16 +3348,16 @@
       <c r="M15" s="5"/>
       <c r="O15" s="5"/>
       <c r="P15" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T15" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X15" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB15" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC15" s="6">
         <f t="shared" si="6"/>
@@ -3337,7 +3374,7 @@
         <v>15</v>
       </c>
       <c r="H16" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L16" s="6">
         <f t="shared" si="0"/>
@@ -3345,16 +3382,16 @@
       <c r="M16" s="5"/>
       <c r="O16" s="5"/>
       <c r="P16" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T16" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X16" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB16" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC16" s="6">
         <f t="shared" si="6"/>
@@ -3371,7 +3408,7 @@
         <v>18</v>
       </c>
       <c r="H17" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L17" s="6">
         <f t="shared" si="0"/>
@@ -3379,16 +3416,16 @@
       <c r="M17" s="5"/>
       <c r="O17" s="5"/>
       <c r="P17" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T17" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X17" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB17" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC17" s="6">
         <f t="shared" si="6"/>
@@ -3405,7 +3442,7 @@
         <v>20</v>
       </c>
       <c r="H18" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L18" s="6">
         <f t="shared" si="0"/>
@@ -3413,16 +3450,16 @@
       <c r="M18" s="5"/>
       <c r="O18" s="5"/>
       <c r="P18" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T18" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X18" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB18" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC18" s="6">
         <f t="shared" si="6"/>
@@ -3439,7 +3476,7 @@
         <v>16</v>
       </c>
       <c r="H19" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L19" s="6">
         <f t="shared" si="0"/>
@@ -3447,16 +3484,16 @@
       <c r="M19" s="5"/>
       <c r="O19" s="5"/>
       <c r="P19" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T19" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X19" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB19" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC19" s="6">
         <f t="shared" si="6"/>
@@ -3473,7 +3510,7 @@
         <v>16</v>
       </c>
       <c r="H20" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L20" s="6">
         <f t="shared" si="0"/>
@@ -3481,16 +3518,16 @@
       <c r="M20" s="5"/>
       <c r="O20" s="5"/>
       <c r="P20" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T20" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X20" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB20" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC20" s="6">
         <f t="shared" si="6"/>
@@ -3507,7 +3544,7 @@
         <v>20</v>
       </c>
       <c r="H21" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L21" s="6">
         <f t="shared" si="0"/>
@@ -3515,16 +3552,16 @@
       <c r="M21" s="5"/>
       <c r="O21" s="5"/>
       <c r="P21" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T21" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X21" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB21" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC21" s="6">
         <f t="shared" si="6"/>
@@ -3541,7 +3578,7 @@
         <v>18</v>
       </c>
       <c r="H22" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L22" s="6">
         <f t="shared" si="0"/>
@@ -3549,16 +3586,16 @@
       <c r="M22" s="5"/>
       <c r="O22" s="5"/>
       <c r="P22" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T22" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X22" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB22" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC22" s="6">
         <f t="shared" si="6"/>
@@ -3575,7 +3612,7 @@
         <v>27</v>
       </c>
       <c r="H23" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L23" s="6">
         <f t="shared" si="0"/>
@@ -3583,16 +3620,16 @@
       <c r="M23" s="5"/>
       <c r="O23" s="5"/>
       <c r="P23" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T23" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X23" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB23" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC23" s="6">
         <f t="shared" si="6"/>
@@ -3609,7 +3646,7 @@
         <v>26</v>
       </c>
       <c r="H24" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L24" s="6">
         <f t="shared" si="0"/>
@@ -3617,16 +3654,16 @@
       <c r="M24" s="5"/>
       <c r="O24" s="5"/>
       <c r="P24" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T24" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X24" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB24" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC24" s="6">
         <f t="shared" si="6"/>
@@ -3643,7 +3680,7 @@
         <v>26</v>
       </c>
       <c r="H25" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L25" s="6">
         <f t="shared" si="0"/>
@@ -3651,16 +3688,16 @@
       <c r="M25" s="5"/>
       <c r="O25" s="5"/>
       <c r="P25" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T25" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X25" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB25" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC25" s="6">
         <f t="shared" si="6"/>
@@ -3677,7 +3714,7 @@
         <v>27</v>
       </c>
       <c r="H26" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L26" s="6">
         <f t="shared" si="0"/>
@@ -3685,16 +3722,16 @@
       <c r="M26" s="5"/>
       <c r="O26" s="5"/>
       <c r="P26" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T26" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X26" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB26" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC26" s="6">
         <f t="shared" si="6"/>
@@ -3711,7 +3748,7 @@
         <v>28</v>
       </c>
       <c r="H27" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L27" s="6">
         <f t="shared" si="0"/>
@@ -3719,16 +3756,16 @@
       <c r="M27" s="5"/>
       <c r="O27" s="5"/>
       <c r="P27" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T27" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X27" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB27" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC27" s="6">
         <f t="shared" si="6"/>
@@ -3745,7 +3782,7 @@
         <v>29</v>
       </c>
       <c r="H28" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L28" s="6">
         <f t="shared" si="0"/>
@@ -3753,16 +3790,16 @@
       <c r="M28" s="5"/>
       <c r="O28" s="5"/>
       <c r="P28" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T28" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X28" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB28" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC28" s="6">
         <f t="shared" si="6"/>
@@ -3779,7 +3816,7 @@
         <v>28</v>
       </c>
       <c r="H29" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="L29" s="6">
         <f t="shared" si="0"/>
@@ -3787,16 +3824,16 @@
       <c r="M29" s="5"/>
       <c r="O29" s="5"/>
       <c r="P29" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T29" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X29" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB29" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC29" s="6">
         <f t="shared" si="6"/>
@@ -3821,16 +3858,16 @@
       <c r="M30" s="5"/>
       <c r="O30" s="5"/>
       <c r="P30" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="T30" s="6">
         <f t="shared" si="5"/>
       </c>
       <c r="X30" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB30" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="AC30" s="6">
         <f t="shared" si="6"/>
@@ -3860,7 +3897,7 @@
         <f t="shared" si="5"/>
       </c>
       <c r="X31" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB31" s="6">
         <f>IFERROR(AVERAGE(AA31:AA31)/D31,"")</f>
@@ -3893,7 +3930,7 @@
         <f t="shared" si="5"/>
       </c>
       <c r="X32" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB32" s="6">
         <f>IFERROR(AVERAGE(AA32:AA32)/D32,"")</f>
@@ -3926,7 +3963,7 @@
         <f t="shared" si="5"/>
       </c>
       <c r="X33" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB33" s="6">
         <f>IFERROR(AVERAGE(AA33:AA33)/D33,"")</f>
@@ -3959,7 +3996,7 @@
         <f t="shared" si="5"/>
       </c>
       <c r="X34" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB34" s="6">
         <f>IFERROR(AVERAGE(AA34:AA34)/D34,"")</f>
@@ -3992,7 +4029,7 @@
         <f t="shared" si="5"/>
       </c>
       <c r="X35" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="AB35" s="6">
         <f>IFERROR(AVERAGE(AA35:AA35)/D35,"")</f>
@@ -5314,12 +5351,14 @@
       </c>
       <c r="N74">
         <f>SUM(N4:N73)</f>
+        <v>23</v>
       </c>
       <c r="O74">
         <f>SUM(O4:O73)</f>
       </c>
       <c r="P74" s="6">
-        <f t="shared" ref="P68:P74" si="15">IFERROR(AVERAGE(M74:O74)/D74,"")</f>
+        <f>IFERROR(AVERAGE(M74:O74)/D74,"")</f>
+        <v>0.0155</v>
       </c>
       <c r="Q74">
         <f>SUM(Q4:Q73)</f>
@@ -5363,7 +5402,7 @@
       </c>
       <c r="AC74" s="6">
         <f>IFERROR(AVERAGE(H74,L74,P74,T74,X74,AB74),"")</f>
-        <v>0.0222</v>
+        <v>0.0205</v>
       </c>
     </row>
   </sheetData>
@@ -5539,27 +5578,27 @@
         <v>22</v>
       </c>
       <c r="H4" s="6">
-        <f t="shared" ref="H4:H49" si="4">IFERROR(AVERAGE(E4:G4)/D4,"")</f>
+        <f t="shared" ref="H4:H49" si="0">IFERROR(AVERAGE(E4:G4)/D4,"")</f>
         <v>0.9565</v>
       </c>
       <c r="L4" s="6">
-        <f t="shared" ref="L4:L50" si="0">IFERROR(AVERAGE(I4:K4)/D4,"")</f>
+        <f t="shared" ref="L4:L50" si="1">IFERROR(AVERAGE(I4:K4)/D4,"")</f>
       </c>
       <c r="N4" s="5">
         <v>26</v>
       </c>
       <c r="P4" s="6">
-        <f t="shared" ref="P4:P49" si="5">IFERROR(AVERAGE(M4:O4)/D4,"")</f>
+        <f t="shared" ref="P4:P49" si="2">IFERROR(AVERAGE(M4:O4)/D4,"")</f>
         <v>1</v>
       </c>
       <c r="T4" s="6">
-        <f t="shared" ref="T4:T50" si="1">IFERROR(AVERAGE(Q4:S4)/D4,"")</f>
+        <f t="shared" ref="T4:T50" si="3">IFERROR(AVERAGE(Q4:S4)/D4,"")</f>
       </c>
       <c r="X4" s="6">
-        <f t="shared" ref="X4:X50" si="2">IFERROR(AVERAGE(U4:W4)/D4,"")</f>
+        <f t="shared" ref="X4:X50" si="4">IFERROR(AVERAGE(U4:W4)/D4,"")</f>
       </c>
       <c r="AB4" s="6">
-        <f t="shared" ref="AB4:AB50" si="3">IFERROR(AVERAGE(Y4:AA4)/D4,"")</f>
+        <f t="shared" ref="AB4:AB50" si="5">IFERROR(AVERAGE(Y4:AA4)/D4,"")</f>
       </c>
       <c r="AC4" s="6">
         <f t="shared" ref="AC4:AC49" si="6">IFERROR(AVERAGE(H4,L4,P4,T4,X4,AB4),"")</f>
@@ -5580,22 +5619,22 @@
         <v>24</v>
       </c>
       <c r="H5" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L5" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P5" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T5" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X5" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB5" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC5" s="6">
         <f t="shared" si="6"/>
@@ -5612,22 +5651,22 @@
         <v>29</v>
       </c>
       <c r="H6" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L6" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P6" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T6" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X6" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB6" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC6" s="6">
         <f t="shared" si="6"/>
@@ -5651,19 +5690,19 @@
         <v>1</v>
       </c>
       <c r="L7" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P7" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T7" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X7" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB7" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC7" s="6">
         <f>IFERROR(AVERAGE(H7,L7,P7,T7,X7,AB7),"")</f>
@@ -5681,22 +5720,22 @@
         <v>19</v>
       </c>
       <c r="H8" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L8" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P8" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T8" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X8" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB8" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC8" s="6">
         <f t="shared" si="6"/>
@@ -5713,22 +5752,22 @@
         <v>22</v>
       </c>
       <c r="H9" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L9" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P9" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T9" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X9" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB9" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC9" s="6">
         <f t="shared" si="6"/>
@@ -5745,22 +5784,22 @@
         <v>19</v>
       </c>
       <c r="H10" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L10" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P10" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T10" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X10" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB10" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC10" s="6">
         <f t="shared" si="6"/>
@@ -5777,22 +5816,22 @@
         <v>18</v>
       </c>
       <c r="H11" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L11" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P11" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T11" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X11" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB11" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC11" s="6">
         <f t="shared" si="6"/>
@@ -5809,22 +5848,22 @@
         <v>17</v>
       </c>
       <c r="H12" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L12" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P12" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T12" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X12" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB12" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC12" s="6">
         <f t="shared" si="6"/>
@@ -5848,19 +5887,19 @@
         <v>1</v>
       </c>
       <c r="L13" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P13" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T13" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X13" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB13" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC13" s="6">
         <f>IFERROR(AVERAGE(H13,L13,P13,T13,X13,AB13),"")</f>
@@ -5878,22 +5917,22 @@
         <v>23</v>
       </c>
       <c r="H14" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L14" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P14" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T14" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X14" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB14" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC14" s="6">
         <f t="shared" si="6"/>
@@ -5910,22 +5949,22 @@
         <v>21</v>
       </c>
       <c r="H15" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L15" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P15" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T15" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X15" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB15" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC15" s="6">
         <f t="shared" si="6"/>
@@ -5942,22 +5981,22 @@
         <v>23</v>
       </c>
       <c r="H16" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L16" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P16" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T16" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X16" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB16" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC16" s="6">
         <f t="shared" si="6"/>
@@ -5974,22 +6013,22 @@
         <v>22</v>
       </c>
       <c r="H17" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L17" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P17" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T17" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X17" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB17" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC17" s="6">
         <f t="shared" si="6"/>
@@ -6006,22 +6045,22 @@
         <v>21</v>
       </c>
       <c r="H18" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L18" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P18" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T18" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X18" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB18" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC18" s="6">
         <f t="shared" si="6"/>
@@ -6038,22 +6077,22 @@
         <v>21</v>
       </c>
       <c r="H19" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L19" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P19" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T19" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X19" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB19" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC19" s="6">
         <f t="shared" si="6"/>
@@ -6070,22 +6109,22 @@
         <v>26</v>
       </c>
       <c r="H20" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L20" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P20" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T20" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X20" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB20" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC20" s="6">
         <f t="shared" si="6"/>
@@ -6102,22 +6141,22 @@
         <v>23</v>
       </c>
       <c r="H21" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L21" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P21" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T21" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X21" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB21" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC21" s="6">
         <f t="shared" si="6"/>
@@ -6134,22 +6173,22 @@
         <v>28</v>
       </c>
       <c r="H22" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L22" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P22" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T22" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X22" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB22" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC22" s="6">
         <f t="shared" si="6"/>
@@ -6166,22 +6205,22 @@
         <v>25</v>
       </c>
       <c r="H23" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L23" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P23" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T23" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X23" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB23" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC23" s="6">
         <f t="shared" si="6"/>
@@ -6198,22 +6237,22 @@
         <v>26</v>
       </c>
       <c r="H24" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L24" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P24" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T24" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X24" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB24" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC24" s="6">
         <f t="shared" si="6"/>
@@ -6230,22 +6269,22 @@
         <v>23</v>
       </c>
       <c r="H25" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L25" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P25" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T25" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X25" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB25" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC25" s="6">
         <f t="shared" si="6"/>
@@ -6262,22 +6301,22 @@
         <v>18</v>
       </c>
       <c r="H26" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L26" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P26" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T26" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X26" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB26" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC26" s="6">
         <f t="shared" si="6"/>
@@ -6294,22 +6333,22 @@
         <v>18</v>
       </c>
       <c r="H27" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L27" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P27" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T27" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X27" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB27" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC27" s="6">
         <f t="shared" si="6"/>
@@ -6326,22 +6365,22 @@
         <v>21</v>
       </c>
       <c r="H28" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L28" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P28" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T28" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X28" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB28" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC28" s="6">
         <f t="shared" si="6"/>
@@ -6358,22 +6397,22 @@
         <v>20</v>
       </c>
       <c r="H29" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L29" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P29" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T29" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X29" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB29" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC29" s="6">
         <f t="shared" si="6"/>
@@ -6390,22 +6429,22 @@
         <v>21</v>
       </c>
       <c r="H30" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L30" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P30" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T30" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X30" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB30" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC30" s="6">
         <f t="shared" si="6"/>
@@ -6422,22 +6461,22 @@
         <v>27</v>
       </c>
       <c r="H31" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L31" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P31" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T31" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X31" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB31" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC31" s="6">
         <f t="shared" si="6"/>
@@ -6461,19 +6500,19 @@
         <v>0.9259</v>
       </c>
       <c r="L32" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P32" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T32" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X32" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB32" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC32" s="6">
         <f>IFERROR(AVERAGE(H32,L32,P32,T32,X32,AB32),"")</f>
@@ -6491,22 +6530,22 @@
         <v>30</v>
       </c>
       <c r="H33" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L33" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P33" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T33" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X33" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB33" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC33" s="6">
         <f t="shared" si="6"/>
@@ -6523,22 +6562,22 @@
         <v>25</v>
       </c>
       <c r="H34" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L34" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P34" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T34" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X34" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB34" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC34" s="6">
         <f t="shared" si="6"/>
@@ -6555,22 +6594,22 @@
         <v>25</v>
       </c>
       <c r="H35" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L35" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P35" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T35" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X35" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB35" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC35" s="6">
         <f t="shared" si="6"/>
@@ -6587,22 +6626,22 @@
         <v>25</v>
       </c>
       <c r="H36" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L36" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P36" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T36" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X36" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB36" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC36" s="6">
         <f t="shared" si="6"/>
@@ -6619,22 +6658,22 @@
         <v>26</v>
       </c>
       <c r="H37" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L37" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P37" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T37" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X37" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB37" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC37" s="6">
         <f t="shared" si="6"/>
@@ -6651,22 +6690,22 @@
         <v>26</v>
       </c>
       <c r="H38" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L38" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P38" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T38" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X38" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB38" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC38" s="6">
         <f t="shared" si="6"/>
@@ -6683,22 +6722,22 @@
         <v>27</v>
       </c>
       <c r="H39" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L39" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P39" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T39" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X39" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB39" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC39" s="6">
         <f t="shared" si="6"/>
@@ -6715,22 +6754,22 @@
         <v>29</v>
       </c>
       <c r="H40" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L40" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P40" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T40" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X40" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB40" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC40" s="6">
         <f t="shared" si="6"/>
@@ -6747,22 +6786,22 @@
         <v>25</v>
       </c>
       <c r="H41" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L41" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P41" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T41" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X41" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB41" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC41" s="6">
         <f t="shared" si="6"/>
@@ -6779,22 +6818,22 @@
         <v>24</v>
       </c>
       <c r="H42" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L42" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P42" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T42" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X42" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB42" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC42" s="6">
         <f t="shared" si="6"/>
@@ -6811,22 +6850,22 @@
         <v>24</v>
       </c>
       <c r="H43" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L43" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P43" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T43" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X43" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB43" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC43" s="6">
         <f t="shared" si="6"/>
@@ -6843,22 +6882,22 @@
         <v>24</v>
       </c>
       <c r="H44" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L44" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P44" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T44" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X44" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB44" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC44" s="6">
         <f t="shared" si="6"/>
@@ -6875,22 +6914,22 @@
         <v>25</v>
       </c>
       <c r="H45" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L45" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P45" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T45" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X45" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB45" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC45" s="6">
         <f t="shared" si="6"/>
@@ -6907,22 +6946,22 @@
         <v>23</v>
       </c>
       <c r="H46" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L46" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P46" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T46" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X46" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB46" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC46" s="6">
         <f t="shared" si="6"/>
@@ -6939,22 +6978,22 @@
         <v>18</v>
       </c>
       <c r="H47" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L47" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P47" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T47" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X47" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB47" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC47" s="6">
         <f t="shared" si="6"/>
@@ -6971,22 +7010,22 @@
         <v>23</v>
       </c>
       <c r="H48" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L48" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P48" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T48" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X48" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB48" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC48" s="6">
         <f t="shared" si="6"/>
@@ -7003,22 +7042,22 @@
         <v>30</v>
       </c>
       <c r="H49" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="0"/>
       </c>
       <c r="L49" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="P49" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
       </c>
       <c r="T49" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="X49" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="AB49" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC49" s="6">
         <f t="shared" si="6"/>
@@ -7056,7 +7095,7 @@
         <f>SUM(K4:K49)</f>
       </c>
       <c r="L50" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
       </c>
       <c r="M50">
         <f>SUM(M4:M49)</f>
@@ -7082,7 +7121,7 @@
         <f>SUM(S4:S49)</f>
       </c>
       <c r="T50" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
       </c>
       <c r="U50">
         <f>SUM(U4:U49)</f>
@@ -7094,7 +7133,7 @@
         <f>SUM(W4:W49)</f>
       </c>
       <c r="X50" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
       </c>
       <c r="Y50">
         <f>SUM(Y4:Y49)</f>
@@ -7106,7 +7145,7 @@
         <f>SUM(AA4:AA49)</f>
       </c>
       <c r="AB50" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
       </c>
       <c r="AC50" s="6">
         <f>IFERROR(AVERAGE(H50,L50,P50,T50,X50,AB50),"")</f>
@@ -10293,7 +10332,7 @@
         <v>696</v>
       </c>
       <c r="E5" s="13">
-        <v>32</v>
+        <v>248</v>
       </c>
       <c r="F5" s="13" t="s">
         <v>261</v>
@@ -10319,7 +10358,7 @@
         <v>1488</v>
       </c>
       <c r="E6" s="13">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F6" s="13" t="s">
         <v>264</v>
@@ -10327,8 +10366,8 @@
       <c r="G6" s="13" t="s">
         <v>265</v>
       </c>
-      <c r="H6" s="14" t="s">
-        <v>263</v>
+      <c r="H6" s="15" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.25">
@@ -10345,13 +10384,13 @@
         <v>1086</v>
       </c>
       <c r="E7" s="13">
-        <v>99</v>
+        <v>26</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="H7" s="14" t="s">
         <v>263</v>
@@ -10371,16 +10410,16 @@
         <v>1243</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>268</v>
-      </c>
-      <c r="H8" s="15" t="s">
         <v>269</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.25">
@@ -10397,42 +10436,42 @@
         <v>638</v>
       </c>
       <c r="E9" s="13">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H9" s="14" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="10" spans="1:8" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
+    <row r="10" spans="1:8" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="17" t="s">
-        <v>272</v>
-      </c>
-      <c r="C10" s="18">
+      <c r="B10" s="18" t="s">
+        <v>273</v>
+      </c>
+      <c r="C10" s="19">
         <v>221</v>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="19">
         <v>5151</v>
       </c>
-      <c r="E10" s="18">
-        <v>187</v>
-      </c>
-      <c r="F10" s="18" t="s">
-        <v>273</v>
-      </c>
-      <c r="G10" s="18" t="s">
-        <v>273</v>
-      </c>
-      <c r="H10" s="19" t="s">
+      <c r="E10" s="19">
+        <v>348</v>
+      </c>
+      <c r="F10" s="19" t="s">
         <v>274</v>
+      </c>
+      <c r="G10" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="H10" s="20" t="s">
+        <v>275</v>
       </c>
     </row>
   </sheetData>

</xml_diff>